<commit_message>
Fix the errors found in the student run-through
Ergoluma's delivery in the 3.4 box, the split-purchase rule (no
contract orders) in 5.4 and Brief C, the approver roles in the
workbook, the 5.4 clause citation, the memo's approver and CC, the
n8n starter's field names, ESCALATE as a policy exception, clause
scoring for Pass cases, and the RFQs' warranty wording.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F3jTzTeVDh4aZxEw8vbSHh
</commit_message>
<xml_diff>
--- a/05-data-analysis/sample-files/purchase-history.xlsx
+++ b/05-data-analysis/sample-files/purchase-history.xlsx
@@ -25133,10 +25133,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="80" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -25231,12 +25231,120 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Approved By</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>The final approver. From RM5,000 to RM50,000 this must be the Head of Procurement, after the HOD</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Received, Open or Cancelled</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Rozita binti Mohd Ariff</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Head of Procurement (also the Procurement HOD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Hafiz bin Kamarudin</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Finance Director (also the Finance HOD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Salmah binti Idris</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Head of Department (HOD), Admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Tan Boon Hock</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Head of Department (HOD), IT</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Farah Nadiah binti Zulkifli</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Head of Department (HOD), Marketing</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Joanne Lee Pei Shan</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Head of Department (HOD), Sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Ganesh a/l Muniandy</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Head of Department (HOD), Warehouse</t>
         </is>
       </c>
     </row>

</xml_diff>